<commit_message>
auto: actualizando historial de vacantes
</commit_message>
<xml_diff>
--- a/nuevas_plazas.xlsx
+++ b/nuevas_plazas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,11 +491,7 @@
           <t>Docente de aula</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Úmbita</t>
@@ -506,10 +502,8 @@
           <t>28/03/2026 a las 08:01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
+      <c r="E2" t="n">
+        <v>63</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -548,11 +542,7 @@
           <t>Docente de aula</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Otanche</t>
@@ -563,10 +553,8 @@
           <t>28/03/2026 a las 08:01</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="E3" t="n">
+        <v>15</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -605,11 +593,7 @@
           <t>Docente de aula</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Ciénega</t>
@@ -620,10 +604,8 @@
           <t>28/03/2026 a las 08:01</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="E4" t="n">
+        <v>19</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -662,11 +644,7 @@
           <t>Docente de aula</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Villa De Leyva</t>
@@ -677,10 +655,8 @@
           <t>28/03/2026 a las 08:01</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="E5" t="n">
+        <v>28</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -719,11 +695,7 @@
           <t>Docente tutor (Planta Temporal PTA)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Támara</t>
@@ -734,10 +706,8 @@
           <t>28/03/2026 a las 08:02</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="E6" t="n">
+        <v>39</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -776,52 +746,103 @@
           <t>Docente de aula</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Girardot</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>28/03/2026 a las 08:03</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>19</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Girardot</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ía de Educación: Girardot</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>I.E. SIMON BOLIVAR</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>I.E. SIMON BOLIVAR SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ón: CL 65 46 A 95</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Docente de aula</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Girardot</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>28/03/2026 a las 08:03</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Girardot</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Cundinamarca</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ía de Educación: Girardot</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Itaguí</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>28/03/2026 a las 08:05</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Itaguí</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ía de Educación: Itaguí</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>I.E. SIMON BOLIVAR</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>I.E. SIMON BOLIVAR SEDE PRINCIPAL</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>ón: CL 65 46 A 95</t>
         </is>

</xml_diff>